<commit_message>
Refactored to publish based usage.
</commit_message>
<xml_diff>
--- a/apps/api/public/templates/avelero-bulk-export-template.xlsx
+++ b/apps/api/public/templates/avelero-bulk-export-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rafmevis/avelero-v2/apps/api/public/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66FFEFAB-E3F1-D744-959D-30290C8665E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEED4F5F-5CDA-5F4B-918C-CA6B7943308C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="21400" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="21360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="90">
   <si>
     <t>Category</t>
   </si>
@@ -78,21 +78,6 @@
   </si>
   <si>
     <t>https://brand.com/image.png</t>
-  </si>
-  <si>
-    <t>Publishing</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Publish status of your product passport</t>
-  </si>
-  <si>
-    <t>Unpublished
-Published
-Archived
-Scheduled</t>
   </si>
   <si>
     <t>Organization</t>
@@ -268,9 +253,6 @@
   </si>
   <si>
     <t>Great organic t-shirt...</t>
-  </si>
-  <si>
-    <t>Unpublished</t>
   </si>
   <si>
     <t>Clothing &gt; T-shirts &amp; Polos &gt; Printed T-shirts</t>
@@ -367,7 +349,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -388,12 +370,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9D2E9"/>
-        <bgColor rgb="FFD9D2E9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFF4CCCC"/>
         <bgColor rgb="FFF4CCCC"/>
       </patternFill>
@@ -402,6 +378,30 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
         <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDAD2EA"/>
+        <bgColor rgb="FFC9DAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDAD2EA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC9DBF9"/>
+        <bgColor rgb="FFD9D2E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC9DBF9"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -482,7 +482,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -490,12 +490,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -505,25 +502,19 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -533,23 +524,41 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFC9DBF9"/>
+      <color rgb="FFDAD2EA"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -762,7 +771,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:F1000"/>
+  <dimension ref="A1:F999"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
@@ -785,7 +794,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="17" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -799,7 +808,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="21"/>
+      <c r="A3" s="18"/>
       <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
@@ -811,7 +820,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="21"/>
+      <c r="A4" s="18"/>
       <c r="B4" s="2" t="s">
         <v>11</v>
       </c>
@@ -823,7 +832,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="21"/>
+      <c r="A5" s="18"/>
       <c r="B5" s="2" t="s">
         <v>2</v>
       </c>
@@ -835,7 +844,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="21"/>
+      <c r="A6" s="18"/>
       <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
@@ -847,267 +856,256 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="28" t="s">
         <v>19</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="4" t="s">
+    </row>
+    <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A8" s="29"/>
+      <c r="B8" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="20" t="s">
+      <c r="C8" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="4" t="s">
+    </row>
+    <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" s="29"/>
+      <c r="B9" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="21"/>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="4" t="s">
+    </row>
+    <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A10" s="30" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="21"/>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>31</v>
+      <c r="D10" s="7" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="31"/>
+      <c r="B11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="C11" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="D11" s="8">
+        <v>115243746</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A12" s="31"/>
+      <c r="B12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="8" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="21"/>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="3" t="s">
+    </row>
+    <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A13" s="31"/>
+      <c r="B13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D12" s="9">
-        <v>115243746</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="21"/>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="D13" s="4" t="s">
+    </row>
+    <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A14" s="31"/>
+      <c r="B14" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="21"/>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="D14" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D14" s="9" t="s">
+    </row>
+    <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A15" s="28" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="21"/>
       <c r="B15" s="2" t="s">
         <v>44</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="8">
+        <v>6.55</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A16" s="29"/>
+      <c r="B16" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="20" t="s">
+      <c r="C16" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="D16" s="9">
+        <v>4223</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A17" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="B17" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D16" s="9">
-        <v>6.55</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="21"/>
-      <c r="B17" s="2" t="s">
+      <c r="C17" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="D17" s="9">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A18" s="31"/>
+      <c r="B18" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D17" s="10">
-        <v>4223</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="22" t="s">
+      <c r="C18" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="D18" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="3" t="s">
+    </row>
+    <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="31"/>
+      <c r="B19" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D18" s="10">
-        <v>792</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A19" s="21"/>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="D19" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="D19" s="10" t="s">
+    </row>
+    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="28" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="21"/>
       <c r="B20" s="2" t="s">
         <v>58</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="29"/>
+      <c r="B21" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="C21" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D21" s="10" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="20" t="s">
+      <c r="E21" s="10"/>
+    </row>
+    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="29"/>
+      <c r="B22" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C22" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="29"/>
+      <c r="B23" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="21"/>
-      <c r="B22" s="2" t="s">
+      <c r="C23" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="D22" s="11" t="s">
+    </row>
+    <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="29"/>
+      <c r="B24" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E22" s="11"/>
-    </row>
-    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A23" s="21"/>
-      <c r="B23" s="2" t="s">
+      <c r="C24" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C23" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A24" s="21"/>
-      <c r="B24" s="2" t="s">
+    </row>
+    <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="29"/>
+      <c r="B25" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="D24" s="3" t="s">
+      <c r="C25" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A25" s="21"/>
-      <c r="B25" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
     <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="21"/>
-      <c r="B26" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>71</v>
-      </c>
+      <c r="D26" s="4"/>
     </row>
     <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D27" s="4"/>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D28" s="4"/>
+      <c r="F28" s="3"/>
     </row>
     <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D29" s="4"/>
-      <c r="F29" s="3"/>
     </row>
     <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D30" s="4"/>
@@ -1205,7 +1203,7 @@
     <row r="61" spans="4:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D61" s="4"/>
     </row>
-    <row r="62" spans="4:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="62" spans="4:4" ht="13" x14ac:dyDescent="0.15">
       <c r="D62" s="4"/>
     </row>
     <row r="63" spans="4:4" ht="13" x14ac:dyDescent="0.15">
@@ -4019,17 +4017,14 @@
     <row r="999" spans="4:4" ht="13" x14ac:dyDescent="0.15">
       <c r="D999" s="4"/>
     </row>
-    <row r="1000" spans="4:4" ht="13" x14ac:dyDescent="0.15">
-      <c r="D1000" s="4"/>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A21:A26"/>
+    <mergeCell ref="A20:A25"/>
     <mergeCell ref="A2:A6"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A11:A15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A10:A14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A17:A19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4040,335 +4035,326 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AC29"/>
+  <dimension ref="A1:AB29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="4" width="18.6640625" customWidth="1"/>
     <col min="5" max="5" width="21.5" customWidth="1"/>
-    <col min="7" max="7" width="19.1640625" customWidth="1"/>
-    <col min="8" max="8" width="17.6640625" customWidth="1"/>
-    <col min="9" max="9" width="17.1640625" customWidth="1"/>
-    <col min="14" max="16" width="15.83203125" customWidth="1"/>
-    <col min="18" max="18" width="16.1640625" customWidth="1"/>
-    <col min="19" max="19" width="15.1640625" customWidth="1"/>
-    <col min="22" max="22" width="16.1640625" customWidth="1"/>
+    <col min="6" max="6" width="19.1640625" customWidth="1"/>
+    <col min="7" max="7" width="17.6640625" customWidth="1"/>
+    <col min="8" max="8" width="17.1640625" customWidth="1"/>
+    <col min="13" max="15" width="15.83203125" customWidth="1"/>
+    <col min="17" max="17" width="16.1640625" customWidth="1"/>
+    <col min="18" max="18" width="15.1640625" customWidth="1"/>
+    <col min="21" max="21" width="16.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="14" x14ac:dyDescent="0.2">
-      <c r="A1" s="23" t="s">
+    <row r="1" spans="1:28" ht="14" x14ac:dyDescent="0.2">
+      <c r="A1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="12" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G1" s="23" t="s">
-        <v>23</v>
-      </c>
+      <c r="G1" s="23"/>
       <c r="H1" s="24"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="26" t="s">
+      <c r="I1" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26"/>
+      <c r="O1" s="26"/>
+      <c r="P1" s="26"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="S1" s="23"/>
+      <c r="T1" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="U1" s="26"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="X1" s="23"/>
+      <c r="Y1" s="23"/>
+      <c r="Z1" s="23"/>
+      <c r="AA1" s="23"/>
+      <c r="AB1" s="24"/>
+    </row>
+    <row r="2" spans="1:28" ht="30" x14ac:dyDescent="0.2">
+      <c r="A2" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="J2" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
-      <c r="O1" s="24"/>
-      <c r="P1" s="24"/>
-      <c r="Q1" s="24"/>
-      <c r="R1" s="25"/>
-      <c r="S1" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="T1" s="24"/>
-      <c r="U1" s="26" t="s">
-        <v>52</v>
-      </c>
-      <c r="V1" s="24"/>
-      <c r="W1" s="25"/>
-      <c r="X1" s="23" t="s">
+      <c r="K2" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L2" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="M2" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="N2" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="O2" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="P2" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q2" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="R2" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="S2" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="T2" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="U2" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="V2" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="W2" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="X2" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y2" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="Y1" s="24"/>
-      <c r="Z1" s="24"/>
-      <c r="AA1" s="24"/>
-      <c r="AB1" s="24"/>
-      <c r="AC1" s="25"/>
-    </row>
-    <row r="2" spans="1:29" ht="30" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F2" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="G2" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="H2" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="I2" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="J2" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="K2" s="13" t="s">
+      <c r="Z2" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="AA2" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="AB2" s="12" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" ht="45" x14ac:dyDescent="0.2">
+      <c r="A3" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="G3" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="I3" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="J3" s="13">
+        <v>115243746</v>
+      </c>
+      <c r="K3" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="L2" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="M2" s="13" t="s">
-        <v>72</v>
-      </c>
-      <c r="N2" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="O2" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="P2" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q2" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="R2" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="S2" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="T2" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="U2" s="14" t="s">
+      <c r="L3" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="M3" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="N3" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="O3" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="P3" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q3" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="R3" s="13">
+        <v>6.55</v>
+      </c>
+      <c r="S3" s="14">
+        <v>4223</v>
+      </c>
+      <c r="T3" s="14">
+        <v>230</v>
+      </c>
+      <c r="U3" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="V2" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="W2" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="X2" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="Y2" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="Z2" s="14" t="s">
+      <c r="V3" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="W3" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="X3" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y3" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z3" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="AA3" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="AA2" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="AB2" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="AC2" s="14" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="3" spans="1:29" ht="45" x14ac:dyDescent="0.2">
-      <c r="A3" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="H3" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="I3" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="J3" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="K3" s="15">
-        <v>115243746</v>
-      </c>
-      <c r="L3" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="M3" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="N3" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="O3" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="P3" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="Q3" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="R3" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="S3" s="15">
-        <v>6.55</v>
-      </c>
-      <c r="T3" s="17">
-        <v>4223</v>
-      </c>
-      <c r="U3" s="17">
-        <v>230</v>
-      </c>
-      <c r="V3" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="W3" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="X3" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="Y3" s="17" t="s">
-        <v>64</v>
-      </c>
-      <c r="Z3" s="15" t="s">
-        <v>94</v>
-      </c>
-      <c r="AA3" s="15" t="s">
-        <v>89</v>
-      </c>
       <c r="AB3" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="AC3" s="18" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="4" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K4" s="19"/>
-      <c r="T4" s="11"/>
-      <c r="V4" s="11"/>
-      <c r="W4" s="11"/>
-      <c r="Y4" s="11"/>
-    </row>
-    <row r="5" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K5" s="19"/>
-    </row>
-    <row r="6" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K6" s="19"/>
-    </row>
-    <row r="7" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K7" s="19"/>
-    </row>
-    <row r="8" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K8" s="19"/>
-    </row>
-    <row r="9" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K9" s="19"/>
-    </row>
-    <row r="10" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K10" s="19"/>
-    </row>
-    <row r="11" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K11" s="19"/>
-    </row>
-    <row r="12" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K12" s="19"/>
-    </row>
-    <row r="13" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K13" s="19"/>
-    </row>
-    <row r="14" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K14" s="19"/>
-    </row>
-    <row r="15" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K15" s="19"/>
-    </row>
-    <row r="16" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K16" s="19"/>
-    </row>
-    <row r="17" spans="11:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K17" s="19"/>
-    </row>
-    <row r="18" spans="11:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K18" s="19"/>
-    </row>
-    <row r="19" spans="11:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K19" s="19"/>
-    </row>
-    <row r="20" spans="11:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K20" s="19"/>
-    </row>
-    <row r="21" spans="11:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K21" s="19"/>
-    </row>
-    <row r="22" spans="11:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K22" s="19"/>
-    </row>
-    <row r="23" spans="11:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K23" s="19"/>
-    </row>
-    <row r="24" spans="11:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K24" s="19"/>
-      <c r="T24" s="11"/>
-      <c r="Y24" s="11"/>
-    </row>
-    <row r="25" spans="11:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K25" s="19"/>
-    </row>
-    <row r="26" spans="11:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K26" s="19"/>
-    </row>
-    <row r="27" spans="11:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K27" s="19"/>
-    </row>
-    <row r="28" spans="11:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K28" s="19"/>
-    </row>
-    <row r="29" spans="11:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="K29" s="19"/>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J4" s="16"/>
+      <c r="S4" s="10"/>
+      <c r="U4" s="10"/>
+      <c r="V4" s="10"/>
+      <c r="X4" s="10"/>
+    </row>
+    <row r="5" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J5" s="16"/>
+    </row>
+    <row r="6" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J6" s="16"/>
+    </row>
+    <row r="7" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J7" s="16"/>
+    </row>
+    <row r="8" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J8" s="16"/>
+    </row>
+    <row r="9" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J9" s="16"/>
+    </row>
+    <row r="10" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J10" s="16"/>
+    </row>
+    <row r="11" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J11" s="16"/>
+    </row>
+    <row r="12" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J12" s="16"/>
+    </row>
+    <row r="13" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J13" s="16"/>
+    </row>
+    <row r="14" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J14" s="16"/>
+    </row>
+    <row r="15" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J15" s="16"/>
+    </row>
+    <row r="16" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J16" s="16"/>
+    </row>
+    <row r="17" spans="10:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J17" s="16"/>
+    </row>
+    <row r="18" spans="10:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J18" s="16"/>
+    </row>
+    <row r="19" spans="10:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J19" s="16"/>
+    </row>
+    <row r="20" spans="10:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J20" s="16"/>
+    </row>
+    <row r="21" spans="10:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J21" s="16"/>
+    </row>
+    <row r="22" spans="10:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J22" s="16"/>
+    </row>
+    <row r="23" spans="10:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J23" s="16"/>
+    </row>
+    <row r="24" spans="10:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J24" s="16"/>
+      <c r="S24" s="10"/>
+      <c r="X24" s="10"/>
+    </row>
+    <row r="25" spans="10:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J25" s="16"/>
+    </row>
+    <row r="26" spans="10:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J26" s="16"/>
+    </row>
+    <row r="27" spans="10:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J27" s="16"/>
+    </row>
+    <row r="28" spans="10:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J28" s="16"/>
+    </row>
+    <row r="29" spans="10:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J29" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="X1:AC1"/>
+    <mergeCell ref="W1:AB1"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="G1:I1"/>
-    <mergeCell ref="J1:R1"/>
-    <mergeCell ref="S1:T1"/>
-    <mergeCell ref="U1:W1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="I1:Q1"/>
+    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="T1:V1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>